<commit_message>
Adding changes - emoved cg executable (too large)
</commit_message>
<xml_diff>
--- a/tutorial/example_5/results-SEP-25-2025.xlsx
+++ b/tutorial/example_5/results-SEP-25-2025.xlsx
@@ -1,19 +1,20 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10913"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10921"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/lagunaperalt1/projects/fpchecker/FPChecker/tutorial/example_5/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{818B9CD2-1830-8442-A99C-31EC7470E049}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FEF64E95-515C-7B46-9131-CB86E4EEA530}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28600" yWindow="2660" windowWidth="23400" windowHeight="17280" xr2:uid="{27EC7522-538B-A648-B33F-CEDE7E825F9B}"/>
+    <workbookView xWindow="20" yWindow="760" windowWidth="30240" windowHeight="17280" activeTab="1" xr2:uid="{27EC7522-538B-A648-B33F-CEDE7E825F9B}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="Sheet2" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="181029" concurrentCalc="0"/>
   <extLst>
@@ -36,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="20" uniqueCount="8">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="30" uniqueCount="14">
   <si>
     <t>line</t>
   </si>
@@ -60,6 +61,24 @@
   </si>
   <si>
     <t>K = 3.848e+02</t>
+  </si>
+  <si>
+    <t>Time</t>
+  </si>
+  <si>
+    <t>Final Residual Error</t>
+  </si>
+  <si>
+    <t>CG (FP32)</t>
+  </si>
+  <si>
+    <t>CG (mixed)</t>
+  </si>
+  <si>
+    <t>CG (FP64)</t>
+  </si>
+  <si>
+    <t>Matrix Cond. Number</t>
   </si>
 </sst>
 </file>
@@ -113,6 +132,2366 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
+  <c:date1904 val="0"/>
+  <c:lang val="en-US"/>
+  <c:roundedCorners val="0"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
+      <c14:style val="102"/>
+    </mc:Choice>
+    <mc:Fallback>
+      <c:style val="2"/>
+    </mc:Fallback>
+  </mc:AlternateContent>
+  <c:chart>
+    <c:title>
+      <c:tx>
+        <c:rich>
+          <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="1600" b="0" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:r>
+              <a:rPr lang="en-US" sz="1600"/>
+              <a:t>Run</a:t>
+            </a:r>
+            <a:r>
+              <a:rPr lang="en-US" sz="1600" baseline="0"/>
+              <a:t> time</a:t>
+            </a:r>
+            <a:endParaRPr lang="en-US" sz="1600"/>
+          </a:p>
+        </c:rich>
+      </c:tx>
+      <c:overlay val="0"/>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+      <c:txPr>
+        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr>
+            <a:defRPr sz="1600" b="0" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="65000"/>
+                  <a:lumOff val="35000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:pPr>
+          <a:endParaRPr lang="en-US"/>
+        </a:p>
+      </c:txPr>
+    </c:title>
+    <c:autoTitleDeleted val="0"/>
+    <c:plotArea>
+      <c:layout/>
+      <c:scatterChart>
+        <c:scatterStyle val="smoothMarker"/>
+        <c:varyColors val="0"/>
+        <c:ser>
+          <c:idx val="0"/>
+          <c:order val="0"/>
+          <c:tx>
+            <c:v>FP32</c:v>
+          </c:tx>
+          <c:spPr>
+            <a:ln w="19050" cap="rnd">
+              <a:solidFill>
+                <a:schemeClr val="accent1"/>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="circle"/>
+            <c:size val="5"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:schemeClr val="accent1"/>
+              </a:solidFill>
+              <a:ln w="9525">
+                <a:solidFill>
+                  <a:schemeClr val="accent1"/>
+                </a:solidFill>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+          </c:marker>
+          <c:xVal>
+            <c:numRef>
+              <c:f>Sheet2!$A$3:$A$8</c:f>
+              <c:numCache>
+                <c:formatCode>0.00E+00</c:formatCode>
+                <c:ptCount val="6"/>
+                <c:pt idx="0">
+                  <c:v>1.04</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>5</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>9</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>41</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>401</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>40000</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:xVal>
+          <c:yVal>
+            <c:numRef>
+              <c:f>Sheet2!$B$3:$B$8</c:f>
+              <c:numCache>
+                <c:formatCode>0.00E+00</c:formatCode>
+                <c:ptCount val="6"/>
+                <c:pt idx="0">
+                  <c:v>4.0535830000000004E-3</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>1.30175E-2</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>1.8331500000000001E-2</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>3.868912E-2</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>0.1225342</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>0.692415</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:yVal>
+          <c:smooth val="1"/>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000000-C59E-304C-86FF-B09D5CCA2467}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:ser>
+          <c:idx val="1"/>
+          <c:order val="1"/>
+          <c:tx>
+            <c:v>Mixed</c:v>
+          </c:tx>
+          <c:spPr>
+            <a:ln w="25400" cap="rnd">
+              <a:solidFill>
+                <a:schemeClr val="accent2"/>
+              </a:solidFill>
+              <a:prstDash val="dash"/>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="circle"/>
+            <c:size val="5"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:schemeClr val="accent2"/>
+              </a:solidFill>
+              <a:ln w="9525">
+                <a:solidFill>
+                  <a:schemeClr val="accent2"/>
+                </a:solidFill>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+          </c:marker>
+          <c:xVal>
+            <c:numRef>
+              <c:f>Sheet2!$A$3:$A$8</c:f>
+              <c:numCache>
+                <c:formatCode>0.00E+00</c:formatCode>
+                <c:ptCount val="6"/>
+                <c:pt idx="0">
+                  <c:v>1.04</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>5</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>9</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>41</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>401</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>40000</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:xVal>
+          <c:yVal>
+            <c:numRef>
+              <c:f>Sheet2!$E$3:$E$8</c:f>
+              <c:numCache>
+                <c:formatCode>0.00E+00</c:formatCode>
+                <c:ptCount val="6"/>
+                <c:pt idx="0">
+                  <c:v>8.9922909999999995E-3</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>3.1001250000000001E-2</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>4.6103249999999998E-2</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>0.1007135</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>0.32686880000000001</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>1.1798070000000001</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:yVal>
+          <c:smooth val="1"/>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000001-C59E-304C-86FF-B09D5CCA2467}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:ser>
+          <c:idx val="2"/>
+          <c:order val="2"/>
+          <c:tx>
+            <c:v>FP64</c:v>
+          </c:tx>
+          <c:spPr>
+            <a:ln w="34925" cap="rnd">
+              <a:solidFill>
+                <a:schemeClr val="bg1">
+                  <a:lumMod val="65000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="circle"/>
+            <c:size val="5"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:schemeClr val="accent3"/>
+              </a:solidFill>
+              <a:ln w="9525">
+                <a:solidFill>
+                  <a:schemeClr val="accent3"/>
+                </a:solidFill>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+          </c:marker>
+          <c:xVal>
+            <c:numRef>
+              <c:f>Sheet2!$A$3:$A$8</c:f>
+              <c:numCache>
+                <c:formatCode>0.00E+00</c:formatCode>
+                <c:ptCount val="6"/>
+                <c:pt idx="0">
+                  <c:v>1.04</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>5</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>9</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>41</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>401</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>40000</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:xVal>
+          <c:yVal>
+            <c:numRef>
+              <c:f>Sheet2!$H$3:$H$8</c:f>
+              <c:numCache>
+                <c:formatCode>0.00E+00</c:formatCode>
+                <c:ptCount val="6"/>
+                <c:pt idx="0">
+                  <c:v>4.4915839999999999E-3</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>1.419429E-2</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>2.0259920000000001E-2</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>4.2010329999999999E-2</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>0.13734750000000001</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>0.48004089999999999</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:yVal>
+          <c:smooth val="1"/>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000002-C59E-304C-86FF-B09D5CCA2467}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:dLbls>
+          <c:showLegendKey val="0"/>
+          <c:showVal val="0"/>
+          <c:showCatName val="0"/>
+          <c:showSerName val="0"/>
+          <c:showPercent val="0"/>
+          <c:showBubbleSize val="0"/>
+        </c:dLbls>
+        <c:axId val="1487044639"/>
+        <c:axId val="1487689295"/>
+      </c:scatterChart>
+      <c:valAx>
+        <c:axId val="1487044639"/>
+        <c:scaling>
+          <c:logBase val="10"/>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="b"/>
+        <c:majorGridlines>
+          <c:spPr>
+            <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="15000"/>
+                  <a:lumOff val="85000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+        </c:majorGridlines>
+        <c:numFmt formatCode="0.00E+00" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+            <a:solidFill>
+              <a:schemeClr val="tx1">
+                <a:lumMod val="25000"/>
+                <a:lumOff val="75000"/>
+              </a:schemeClr>
+            </a:solidFill>
+            <a:round/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="1400" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="en-US"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="1487689295"/>
+        <c:crosses val="autoZero"/>
+        <c:crossBetween val="midCat"/>
+      </c:valAx>
+      <c:valAx>
+        <c:axId val="1487689295"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="l"/>
+        <c:majorGridlines>
+          <c:spPr>
+            <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="15000"/>
+                  <a:lumOff val="85000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+        </c:majorGridlines>
+        <c:numFmt formatCode="0.00E+00" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+            <a:solidFill>
+              <a:schemeClr val="tx1">
+                <a:lumMod val="25000"/>
+                <a:lumOff val="75000"/>
+              </a:schemeClr>
+            </a:solidFill>
+            <a:round/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="1200" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="en-US"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="1487044639"/>
+        <c:crosses val="autoZero"/>
+        <c:crossBetween val="midCat"/>
+      </c:valAx>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+    </c:plotArea>
+    <c:legend>
+      <c:legendPos val="b"/>
+      <c:layout>
+        <c:manualLayout>
+          <c:xMode val="edge"/>
+          <c:yMode val="edge"/>
+          <c:x val="0.13618560179977501"/>
+          <c:y val="0.14585770861482555"/>
+          <c:w val="0.15441437007874015"/>
+          <c:h val="0.18668667008339937"/>
+        </c:manualLayout>
+      </c:layout>
+      <c:overlay val="0"/>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+      <c:txPr>
+        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr>
+            <a:defRPr sz="1400" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="65000"/>
+                  <a:lumOff val="35000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:pPr>
+          <a:endParaRPr lang="en-US"/>
+        </a:p>
+      </c:txPr>
+    </c:legend>
+    <c:plotVisOnly val="1"/>
+    <c:dispBlanksAs val="gap"/>
+    <c:showDLblsOverMax val="0"/>
+    <c:extLst>
+      <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
+        <c16r3:dataDisplayOptions16>
+          <c16r3:dispNaAsBlank val="1"/>
+        </c16r3:dataDisplayOptions16>
+      </c:ext>
+    </c:extLst>
+  </c:chart>
+  <c:spPr>
+    <a:solidFill>
+      <a:schemeClr val="bg1"/>
+    </a:solidFill>
+    <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+      <a:solidFill>
+        <a:schemeClr val="tx1">
+          <a:lumMod val="15000"/>
+          <a:lumOff val="85000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:round/>
+    </a:ln>
+    <a:effectLst/>
+  </c:spPr>
+  <c:txPr>
+    <a:bodyPr/>
+    <a:lstStyle/>
+    <a:p>
+      <a:pPr>
+        <a:defRPr/>
+      </a:pPr>
+      <a:endParaRPr lang="en-US"/>
+    </a:p>
+  </c:txPr>
+  <c:printSettings>
+    <c:headerFooter/>
+    <c:pageMargins b="0.75" l="0.7" r="0.7" t="0.75" header="0.3" footer="0.3"/>
+    <c:pageSetup/>
+  </c:printSettings>
+</c:chartSpace>
+</file>
+
+<file path=xl/charts/chart2.xml><?xml version="1.0" encoding="utf-8"?>
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
+  <c:date1904 val="0"/>
+  <c:lang val="en-US"/>
+  <c:roundedCorners val="0"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
+      <c14:style val="102"/>
+    </mc:Choice>
+    <mc:Fallback>
+      <c:style val="2"/>
+    </mc:Fallback>
+  </mc:AlternateContent>
+  <c:chart>
+    <c:title>
+      <c:tx>
+        <c:rich>
+          <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="1600" b="0" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:r>
+              <a:rPr lang="en-US" sz="1600"/>
+              <a:t>Final</a:t>
+            </a:r>
+            <a:r>
+              <a:rPr lang="en-US" sz="1600" baseline="0"/>
+              <a:t> Residual Error</a:t>
+            </a:r>
+            <a:endParaRPr lang="en-US" sz="1600"/>
+          </a:p>
+        </c:rich>
+      </c:tx>
+      <c:overlay val="0"/>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+      <c:txPr>
+        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr>
+            <a:defRPr sz="1600" b="0" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="65000"/>
+                  <a:lumOff val="35000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:pPr>
+          <a:endParaRPr lang="en-US"/>
+        </a:p>
+      </c:txPr>
+    </c:title>
+    <c:autoTitleDeleted val="0"/>
+    <c:plotArea>
+      <c:layout/>
+      <c:scatterChart>
+        <c:scatterStyle val="smoothMarker"/>
+        <c:varyColors val="0"/>
+        <c:ser>
+          <c:idx val="0"/>
+          <c:order val="0"/>
+          <c:tx>
+            <c:v>FP32</c:v>
+          </c:tx>
+          <c:spPr>
+            <a:ln w="19050" cap="rnd">
+              <a:solidFill>
+                <a:schemeClr val="accent1"/>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="circle"/>
+            <c:size val="5"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:schemeClr val="accent1"/>
+              </a:solidFill>
+              <a:ln w="9525">
+                <a:solidFill>
+                  <a:schemeClr val="accent1"/>
+                </a:solidFill>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+          </c:marker>
+          <c:xVal>
+            <c:numRef>
+              <c:f>Sheet2!$A$3:$A$8</c:f>
+              <c:numCache>
+                <c:formatCode>0.00E+00</c:formatCode>
+                <c:ptCount val="6"/>
+                <c:pt idx="0">
+                  <c:v>1.04</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>5</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>9</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>41</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>401</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>40000</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:xVal>
+          <c:yVal>
+            <c:numRef>
+              <c:f>Sheet2!$C$3:$C$8</c:f>
+              <c:numCache>
+                <c:formatCode>0.00E+00</c:formatCode>
+                <c:ptCount val="6"/>
+                <c:pt idx="0">
+                  <c:v>2.215124E-6</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>3.043569E-5</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>1.7603870000000001E-5</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>3.5679300000000002E-5</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>6.9037250000000003E-4</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>0.27591149999999998</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:yVal>
+          <c:smooth val="1"/>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000000-0A66-D343-958B-EB90D781243B}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:ser>
+          <c:idx val="1"/>
+          <c:order val="1"/>
+          <c:tx>
+            <c:v>Mixed</c:v>
+          </c:tx>
+          <c:spPr>
+            <a:ln w="25400" cap="rnd">
+              <a:solidFill>
+                <a:schemeClr val="accent2"/>
+              </a:solidFill>
+              <a:prstDash val="dash"/>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="circle"/>
+            <c:size val="5"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:schemeClr val="accent2"/>
+              </a:solidFill>
+              <a:ln w="9525">
+                <a:solidFill>
+                  <a:schemeClr val="accent2"/>
+                </a:solidFill>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+          </c:marker>
+          <c:xVal>
+            <c:numRef>
+              <c:f>Sheet2!$A$3:$A$8</c:f>
+              <c:numCache>
+                <c:formatCode>0.00E+00</c:formatCode>
+                <c:ptCount val="6"/>
+                <c:pt idx="0">
+                  <c:v>1.04</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>5</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>9</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>41</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>401</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>40000</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:xVal>
+          <c:yVal>
+            <c:numRef>
+              <c:f>Sheet2!$F$3:$F$8</c:f>
+              <c:numCache>
+                <c:formatCode>0.00E+00</c:formatCode>
+                <c:ptCount val="6"/>
+                <c:pt idx="0">
+                  <c:v>2.215124E-6</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>3.0833059999999999E-5</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>1.771211E-5</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>3.6303929999999999E-5</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>6.4280049999999997E-4</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>0.22929340000000001</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:yVal>
+          <c:smooth val="1"/>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000001-0A66-D343-958B-EB90D781243B}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:ser>
+          <c:idx val="2"/>
+          <c:order val="2"/>
+          <c:tx>
+            <c:v>FP64</c:v>
+          </c:tx>
+          <c:spPr>
+            <a:ln w="34925" cap="rnd">
+              <a:solidFill>
+                <a:schemeClr val="bg1">
+                  <a:lumMod val="65000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="circle"/>
+            <c:size val="5"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:schemeClr val="accent3"/>
+              </a:solidFill>
+              <a:ln w="9525">
+                <a:solidFill>
+                  <a:schemeClr val="accent3"/>
+                </a:solidFill>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+          </c:marker>
+          <c:xVal>
+            <c:numRef>
+              <c:f>Sheet2!$A$3:$A$8</c:f>
+              <c:numCache>
+                <c:formatCode>0.00E+00</c:formatCode>
+                <c:ptCount val="6"/>
+                <c:pt idx="0">
+                  <c:v>1.04</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>5</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>9</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>41</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>401</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>40000</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:xVal>
+          <c:yVal>
+            <c:numRef>
+              <c:f>Sheet2!$I$3:$I$8</c:f>
+              <c:numCache>
+                <c:formatCode>0.00E+00</c:formatCode>
+                <c:ptCount val="6"/>
+                <c:pt idx="0">
+                  <c:v>2.2192650000000002E-6</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>3.0431839999999998E-5</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>1.6136270000000001E-5</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>3.0435629999999999E-5</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>3.1337410000000003E-5</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>1.9073489999999998E-6</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:yVal>
+          <c:smooth val="1"/>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000002-0A66-D343-958B-EB90D781243B}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:dLbls>
+          <c:showLegendKey val="0"/>
+          <c:showVal val="0"/>
+          <c:showCatName val="0"/>
+          <c:showSerName val="0"/>
+          <c:showPercent val="0"/>
+          <c:showBubbleSize val="0"/>
+        </c:dLbls>
+        <c:axId val="947275743"/>
+        <c:axId val="22271695"/>
+      </c:scatterChart>
+      <c:valAx>
+        <c:axId val="947275743"/>
+        <c:scaling>
+          <c:logBase val="10"/>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="b"/>
+        <c:majorGridlines>
+          <c:spPr>
+            <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="15000"/>
+                  <a:lumOff val="85000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+        </c:majorGridlines>
+        <c:numFmt formatCode="0.00E+00" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+            <a:solidFill>
+              <a:schemeClr val="tx1">
+                <a:lumMod val="25000"/>
+                <a:lumOff val="75000"/>
+              </a:schemeClr>
+            </a:solidFill>
+            <a:round/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="1400" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="en-US"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="22271695"/>
+        <c:crosses val="autoZero"/>
+        <c:crossBetween val="midCat"/>
+      </c:valAx>
+      <c:valAx>
+        <c:axId val="22271695"/>
+        <c:scaling>
+          <c:logBase val="10"/>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="l"/>
+        <c:majorGridlines>
+          <c:spPr>
+            <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="15000"/>
+                  <a:lumOff val="85000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+        </c:majorGridlines>
+        <c:numFmt formatCode="0.00E+00" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+            <a:solidFill>
+              <a:schemeClr val="tx1">
+                <a:lumMod val="25000"/>
+                <a:lumOff val="75000"/>
+              </a:schemeClr>
+            </a:solidFill>
+            <a:round/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="1200" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="en-US"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="947275743"/>
+        <c:crosses val="autoZero"/>
+        <c:crossBetween val="midCat"/>
+      </c:valAx>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+    </c:plotArea>
+    <c:legend>
+      <c:legendPos val="b"/>
+      <c:layout>
+        <c:manualLayout>
+          <c:xMode val="edge"/>
+          <c:yMode val="edge"/>
+          <c:x val="0.11266991123596988"/>
+          <c:y val="0.22283491303824715"/>
+          <c:w val="0.15829172107255435"/>
+          <c:h val="0.24081173214978008"/>
+        </c:manualLayout>
+      </c:layout>
+      <c:overlay val="0"/>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+      <c:txPr>
+        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr>
+            <a:defRPr sz="1400" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="65000"/>
+                  <a:lumOff val="35000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:pPr>
+          <a:endParaRPr lang="en-US"/>
+        </a:p>
+      </c:txPr>
+    </c:legend>
+    <c:plotVisOnly val="1"/>
+    <c:dispBlanksAs val="gap"/>
+    <c:showDLblsOverMax val="0"/>
+    <c:extLst>
+      <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
+        <c16r3:dataDisplayOptions16>
+          <c16r3:dispNaAsBlank val="1"/>
+        </c16r3:dataDisplayOptions16>
+      </c:ext>
+    </c:extLst>
+  </c:chart>
+  <c:spPr>
+    <a:solidFill>
+      <a:schemeClr val="bg1"/>
+    </a:solidFill>
+    <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+      <a:solidFill>
+        <a:schemeClr val="tx1">
+          <a:lumMod val="15000"/>
+          <a:lumOff val="85000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:round/>
+    </a:ln>
+    <a:effectLst/>
+  </c:spPr>
+  <c:txPr>
+    <a:bodyPr/>
+    <a:lstStyle/>
+    <a:p>
+      <a:pPr>
+        <a:defRPr/>
+      </a:pPr>
+      <a:endParaRPr lang="en-US"/>
+    </a:p>
+  </c:txPr>
+  <c:printSettings>
+    <c:headerFooter/>
+    <c:pageMargins b="0.75" l="0.7" r="0.7" t="0.75" header="0.3" footer="0.3"/>
+    <c:pageSetup/>
+  </c:printSettings>
+</c:chartSpace>
+</file>
+
+<file path=xl/charts/colors1.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:colorStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" meth="cycle" id="10">
+  <a:schemeClr val="accent1"/>
+  <a:schemeClr val="accent2"/>
+  <a:schemeClr val="accent3"/>
+  <a:schemeClr val="accent4"/>
+  <a:schemeClr val="accent5"/>
+  <a:schemeClr val="accent6"/>
+  <cs:variation/>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+    <a:lumOff val="20000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+    <a:lumOff val="40000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+    <a:lumOff val="30000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+    <a:lumOff val="50000"/>
+  </cs:variation>
+</cs:colorStyle>
+</file>
+
+<file path=xl/charts/colors2.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:colorStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" meth="cycle" id="10">
+  <a:schemeClr val="accent1"/>
+  <a:schemeClr val="accent2"/>
+  <a:schemeClr val="accent3"/>
+  <a:schemeClr val="accent4"/>
+  <a:schemeClr val="accent5"/>
+  <a:schemeClr val="accent6"/>
+  <cs:variation/>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+    <a:lumOff val="20000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+    <a:lumOff val="40000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+    <a:lumOff val="30000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+    <a:lumOff val="50000"/>
+  </cs:variation>
+</cs:colorStyle>
+</file>
+
+<file path=xl/charts/style1.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="240">
+  <cs:axisTitle>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1000" kern="1200"/>
+  </cs:axisTitle>
+  <cs:categoryAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="25000"/>
+            <a:lumOff val="75000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:categoryAxis>
+  <cs:chartArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="bg1"/>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="1000" kern="1200"/>
+  </cs:chartArea>
+  <cs:dataLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="75000"/>
+        <a:lumOff val="25000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataLabel>
+  <cs:dataLabelCallout>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln>
+        <a:solidFill>
+          <a:schemeClr val="dk1">
+            <a:lumMod val="25000"/>
+            <a:lumOff val="75000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+    <cs:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="clip" horzOverflow="clip" vert="horz" wrap="square" lIns="36576" tIns="18288" rIns="36576" bIns="18288" anchor="ctr" anchorCtr="1">
+      <a:spAutoFit/>
+    </cs:bodyPr>
+  </cs:dataLabelCallout>
+  <cs:dataPoint>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:dataPoint>
+  <cs:dataPoint3D>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:dataPoint3D>
+  <cs:dataPointLine>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="19050" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointLine>
+  <cs:dataPointMarker>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointMarker>
+  <cs:dataPointMarkerLayout symbol="circle" size="5"/>
+  <cs:dataPointWireframe>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointWireframe>
+  <cs:dataTable>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataTable>
+  <cs:downBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="dk1">
+          <a:lumMod val="75000"/>
+          <a:lumOff val="25000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:downBar>
+  <cs:dropLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dropLine>
+  <cs:errorBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:errorBar>
+  <cs:floor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln>
+        <a:noFill/>
+      </a:ln>
+    </cs:spPr>
+  </cs:floor>
+  <cs:gridlineMajor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMajor>
+  <cs:gridlineMinor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="5000"/>
+            <a:lumOff val="95000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMinor>
+  <cs:hiLoLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="50000"/>
+            <a:lumOff val="50000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:hiLoLine>
+  <cs:leaderLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:leaderLine>
+  <cs:legend>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:legend>
+  <cs:plotArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea>
+  <cs:plotArea3D mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea3D>
+  <cs:seriesAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:seriesAxis>
+  <cs:seriesLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:seriesLine>
+  <cs:title>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1400" b="0" kern="1200" spc="0" baseline="0"/>
+  </cs:title>
+  <cs:trendline>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="19050" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:prstDash val="sysDot"/>
+      </a:ln>
+    </cs:spPr>
+  </cs:trendline>
+  <cs:trendlineLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:trendlineLabel>
+  <cs:upBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:upBar>
+  <cs:valueAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="25000"/>
+            <a:lumOff val="75000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:valueAxis>
+  <cs:wall>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln>
+        <a:noFill/>
+      </a:ln>
+    </cs:spPr>
+  </cs:wall>
+</cs:chartStyle>
+</file>
+
+<file path=xl/charts/style2.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="240">
+  <cs:axisTitle>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1000" kern="1200"/>
+  </cs:axisTitle>
+  <cs:categoryAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="25000"/>
+            <a:lumOff val="75000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:categoryAxis>
+  <cs:chartArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="bg1"/>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="1000" kern="1200"/>
+  </cs:chartArea>
+  <cs:dataLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="75000"/>
+        <a:lumOff val="25000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataLabel>
+  <cs:dataLabelCallout>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln>
+        <a:solidFill>
+          <a:schemeClr val="dk1">
+            <a:lumMod val="25000"/>
+            <a:lumOff val="75000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+    <cs:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="clip" horzOverflow="clip" vert="horz" wrap="square" lIns="36576" tIns="18288" rIns="36576" bIns="18288" anchor="ctr" anchorCtr="1">
+      <a:spAutoFit/>
+    </cs:bodyPr>
+  </cs:dataLabelCallout>
+  <cs:dataPoint>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:dataPoint>
+  <cs:dataPoint3D>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:dataPoint3D>
+  <cs:dataPointLine>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="19050" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointLine>
+  <cs:dataPointMarker>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointMarker>
+  <cs:dataPointMarkerLayout symbol="circle" size="5"/>
+  <cs:dataPointWireframe>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointWireframe>
+  <cs:dataTable>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataTable>
+  <cs:downBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="dk1">
+          <a:lumMod val="75000"/>
+          <a:lumOff val="25000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:downBar>
+  <cs:dropLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dropLine>
+  <cs:errorBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:errorBar>
+  <cs:floor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln>
+        <a:noFill/>
+      </a:ln>
+    </cs:spPr>
+  </cs:floor>
+  <cs:gridlineMajor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMajor>
+  <cs:gridlineMinor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="5000"/>
+            <a:lumOff val="95000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMinor>
+  <cs:hiLoLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="50000"/>
+            <a:lumOff val="50000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:hiLoLine>
+  <cs:leaderLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:leaderLine>
+  <cs:legend>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:legend>
+  <cs:plotArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea>
+  <cs:plotArea3D mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea3D>
+  <cs:seriesAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:seriesAxis>
+  <cs:seriesLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:seriesLine>
+  <cs:title>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1400" b="0" kern="1200" spc="0" baseline="0"/>
+  </cs:title>
+  <cs:trendline>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="19050" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:prstDash val="sysDot"/>
+      </a:ln>
+    </cs:spPr>
+  </cs:trendline>
+  <cs:trendlineLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:trendlineLabel>
+  <cs:upBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:upBar>
+  <cs:valueAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="25000"/>
+            <a:lumOff val="75000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:valueAxis>
+  <cs:wall>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln>
+        <a:noFill/>
+      </a:ln>
+    </cs:spPr>
+  </cs:wall>
+</cs:chartStyle>
+</file>
+
+<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>10</xdr:col>
+      <xdr:colOff>368300</xdr:colOff>
+      <xdr:row>0</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>19</xdr:col>
+      <xdr:colOff>571500</xdr:colOff>
+      <xdr:row>17</xdr:row>
+      <xdr:rowOff>63500</xdr:rowOff>
+    </xdr:to>
+    <xdr:graphicFrame macro="">
+      <xdr:nvGraphicFramePr>
+        <xdr:cNvPr id="5" name="Chart 4">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{06DAB0B4-DECA-4AFD-133A-8BC9BC70082A}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvGraphicFramePr/>
+      </xdr:nvGraphicFramePr>
+      <xdr:xfrm>
+        <a:off x="0" y="0"/>
+        <a:ext cx="0" cy="0"/>
+      </xdr:xfrm>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+        </a:graphicData>
+      </a:graphic>
+    </xdr:graphicFrame>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>10</xdr:col>
+      <xdr:colOff>381000</xdr:colOff>
+      <xdr:row>17</xdr:row>
+      <xdr:rowOff>171450</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>19</xdr:col>
+      <xdr:colOff>533400</xdr:colOff>
+      <xdr:row>36</xdr:row>
+      <xdr:rowOff>50800</xdr:rowOff>
+    </xdr:to>
+    <xdr:graphicFrame macro="">
+      <xdr:nvGraphicFramePr>
+        <xdr:cNvPr id="6" name="Chart 5">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{C112A35E-F5A7-463A-6FE9-D2E66991B1C2}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvGraphicFramePr/>
+      </xdr:nvGraphicFramePr>
+      <xdr:xfrm>
+        <a:off x="0" y="0"/>
+        <a:ext cx="0" cy="0"/>
+      </xdr:xfrm>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId2"/>
+        </a:graphicData>
+      </a:graphic>
+    </xdr:graphicFrame>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -810,4 +3189,191 @@
   </sortState>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1317E7BD-FC47-9C46-B2C3-C42C2306F055}">
+  <dimension ref="A1:I8"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="1" max="1" width="20.1640625" customWidth="1"/>
+    <col min="3" max="3" width="17.83203125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="B1" t="s">
+        <v>10</v>
+      </c>
+      <c r="E1" t="s">
+        <v>11</v>
+      </c>
+      <c r="H1" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="2" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A2" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="B2" t="s">
+        <v>8</v>
+      </c>
+      <c r="C2" t="s">
+        <v>9</v>
+      </c>
+      <c r="E2" t="s">
+        <v>8</v>
+      </c>
+      <c r="F2" t="s">
+        <v>9</v>
+      </c>
+      <c r="H2" t="s">
+        <v>8</v>
+      </c>
+      <c r="I2" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="3" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A3" s="1">
+        <v>1.04</v>
+      </c>
+      <c r="B3" s="1">
+        <v>4.0535830000000004E-3</v>
+      </c>
+      <c r="C3" s="1">
+        <v>2.215124E-6</v>
+      </c>
+      <c r="E3" s="1">
+        <v>8.9922909999999995E-3</v>
+      </c>
+      <c r="F3" s="1">
+        <v>2.215124E-6</v>
+      </c>
+      <c r="H3" s="1">
+        <v>4.4915839999999999E-3</v>
+      </c>
+      <c r="I3" s="1">
+        <v>2.2192650000000002E-6</v>
+      </c>
+    </row>
+    <row r="4" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A4" s="1">
+        <v>5</v>
+      </c>
+      <c r="B4" s="1">
+        <v>1.30175E-2</v>
+      </c>
+      <c r="C4" s="1">
+        <v>3.043569E-5</v>
+      </c>
+      <c r="E4" s="1">
+        <v>3.1001250000000001E-2</v>
+      </c>
+      <c r="F4" s="1">
+        <v>3.0833059999999999E-5</v>
+      </c>
+      <c r="H4" s="1">
+        <v>1.419429E-2</v>
+      </c>
+      <c r="I4" s="1">
+        <v>3.0431839999999998E-5</v>
+      </c>
+    </row>
+    <row r="5" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A5" s="1">
+        <v>9</v>
+      </c>
+      <c r="B5" s="1">
+        <v>1.8331500000000001E-2</v>
+      </c>
+      <c r="C5" s="1">
+        <v>1.7603870000000001E-5</v>
+      </c>
+      <c r="E5" s="1">
+        <v>4.6103249999999998E-2</v>
+      </c>
+      <c r="F5" s="1">
+        <v>1.771211E-5</v>
+      </c>
+      <c r="H5" s="1">
+        <v>2.0259920000000001E-2</v>
+      </c>
+      <c r="I5" s="1">
+        <v>1.6136270000000001E-5</v>
+      </c>
+    </row>
+    <row r="6" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A6" s="1">
+        <v>41</v>
+      </c>
+      <c r="B6" s="1">
+        <v>3.868912E-2</v>
+      </c>
+      <c r="C6" s="1">
+        <v>3.5679300000000002E-5</v>
+      </c>
+      <c r="E6" s="1">
+        <v>0.1007135</v>
+      </c>
+      <c r="F6" s="1">
+        <v>3.6303929999999999E-5</v>
+      </c>
+      <c r="H6" s="1">
+        <v>4.2010329999999999E-2</v>
+      </c>
+      <c r="I6" s="1">
+        <v>3.0435629999999999E-5</v>
+      </c>
+    </row>
+    <row r="7" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A7" s="1">
+        <v>401</v>
+      </c>
+      <c r="B7" s="1">
+        <v>0.1225342</v>
+      </c>
+      <c r="C7" s="1">
+        <v>6.9037250000000003E-4</v>
+      </c>
+      <c r="E7" s="1">
+        <v>0.32686880000000001</v>
+      </c>
+      <c r="F7" s="1">
+        <v>6.4280049999999997E-4</v>
+      </c>
+      <c r="H7" s="1">
+        <v>0.13734750000000001</v>
+      </c>
+      <c r="I7" s="1">
+        <v>3.1337410000000003E-5</v>
+      </c>
+    </row>
+    <row r="8" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A8" s="1">
+        <v>40000</v>
+      </c>
+      <c r="B8" s="1">
+        <v>0.692415</v>
+      </c>
+      <c r="C8" s="1">
+        <v>0.27591149999999998</v>
+      </c>
+      <c r="E8" s="1">
+        <v>1.1798070000000001</v>
+      </c>
+      <c r="F8" s="1">
+        <v>0.22929340000000001</v>
+      </c>
+      <c r="H8" s="1">
+        <v>0.48004089999999999</v>
+      </c>
+      <c r="I8" s="1">
+        <v>1.9073489999999998E-6</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <drawing r:id="rId1"/>
+</worksheet>
 </file>
</xml_diff>